<commit_message>
Update partner tracking workbook
</commit_message>
<xml_diff>
--- a/data/partner/Focus Partner Tracking BR.xlsx
+++ b/data/partner/Focus Partner Tracking BR.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mrovere/Library/CloudStorage/GoogleDrive-marcelo@mrovere.com/Other computers/My MacBook Pro/Tenable - geral/Internal - Tenable/Canais/2026 news/EM Cert/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mrovere/Documents/Codex/2026-05-29/acesso-o-google-drive-e-analise/mrovere-treino-push/data/partner/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8134D0E-2241-0747-815D-CB9C2EC72110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -574,14 +574,11 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -594,19 +591,14 @@
     <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="11">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFCE5CD"/>
-          <bgColor rgb="FFFCE5CD"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -636,6 +628,14 @@
         <patternFill patternType="solid">
           <fgColor rgb="FFC9DAF8"/>
           <bgColor rgb="FFC9DAF8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFCE5CD"/>
+          <bgColor rgb="FFFCE5CD"/>
         </patternFill>
       </fill>
     </dxf>
@@ -945,38 +945,38 @@
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
-      <c r="F1" s="31" t="s">
+      <c r="F1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="30"/>
-      <c r="K1" s="30"/>
-      <c r="L1" s="30"/>
-      <c r="M1" s="30"/>
-      <c r="N1" s="30"/>
-      <c r="O1" s="30"/>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="30"/>
-      <c r="R1" s="30"/>
-      <c r="S1" s="30"/>
-      <c r="T1" s="29"/>
-      <c r="U1" s="31" t="s">
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
+      <c r="O1" s="29"/>
+      <c r="P1" s="29"/>
+      <c r="Q1" s="29"/>
+      <c r="R1" s="29"/>
+      <c r="S1" s="29"/>
+      <c r="T1" s="30"/>
+      <c r="U1" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="V1" s="29"/>
-      <c r="W1" s="31" t="s">
+      <c r="V1" s="30"/>
+      <c r="W1" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="X1" s="30"/>
-      <c r="Y1" s="30"/>
-      <c r="Z1" s="30"/>
-      <c r="AA1" s="30"/>
-      <c r="AB1" s="30"/>
-      <c r="AC1" s="30"/>
-      <c r="AD1" s="30"/>
-      <c r="AE1" s="29"/>
+      <c r="X1" s="29"/>
+      <c r="Y1" s="29"/>
+      <c r="Z1" s="29"/>
+      <c r="AA1" s="29"/>
+      <c r="AB1" s="29"/>
+      <c r="AC1" s="29"/>
+      <c r="AD1" s="29"/>
+      <c r="AE1" s="30"/>
     </row>
     <row r="2" spans="1:31" ht="13" x14ac:dyDescent="0.15">
       <c r="A2" s="2"/>
@@ -984,25 +984,25 @@
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="4"/>
-      <c r="F2" s="32" t="s">
+      <c r="F2" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
-      <c r="K2" s="30"/>
-      <c r="L2" s="30"/>
-      <c r="M2" s="29"/>
-      <c r="N2" s="33" t="s">
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="29"/>
+      <c r="K2" s="29"/>
+      <c r="L2" s="29"/>
+      <c r="M2" s="30"/>
+      <c r="N2" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="O2" s="30"/>
-      <c r="P2" s="30"/>
-      <c r="Q2" s="30"/>
-      <c r="R2" s="30"/>
-      <c r="S2" s="30"/>
-      <c r="T2" s="29"/>
+      <c r="O2" s="29"/>
+      <c r="P2" s="29"/>
+      <c r="Q2" s="29"/>
+      <c r="R2" s="29"/>
+      <c r="S2" s="29"/>
+      <c r="T2" s="30"/>
       <c r="U2" s="5" t="s">
         <v>5</v>
       </c>
@@ -1012,18 +1012,18 @@
       <c r="W2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="X2" s="34" t="s">
+      <c r="X2" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="Y2" s="30"/>
-      <c r="Z2" s="30"/>
-      <c r="AA2" s="29"/>
-      <c r="AB2" s="35" t="s">
+      <c r="Y2" s="29"/>
+      <c r="Z2" s="29"/>
+      <c r="AA2" s="30"/>
+      <c r="AB2" s="34" t="s">
         <v>9</v>
       </c>
-      <c r="AC2" s="30"/>
-      <c r="AD2" s="30"/>
-      <c r="AE2" s="29"/>
+      <c r="AC2" s="29"/>
+      <c r="AD2" s="29"/>
+      <c r="AE2" s="30"/>
     </row>
     <row r="3" spans="1:31" ht="13" x14ac:dyDescent="0.15">
       <c r="A3" s="8" t="s">
@@ -1125,10 +1125,10 @@
       <c r="F4" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="G4" s="28" t="s">
+      <c r="G4" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="H4" s="29"/>
+      <c r="H4" s="30"/>
       <c r="I4" s="20" t="s">
         <v>28</v>
       </c>
@@ -1147,15 +1147,15 @@
       <c r="N4" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="O4" s="28" t="s">
+      <c r="O4" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="P4" s="29"/>
-      <c r="Q4" s="28" t="s">
+      <c r="P4" s="30"/>
+      <c r="Q4" s="35" t="s">
         <v>30</v>
       </c>
-      <c r="R4" s="30"/>
-      <c r="S4" s="29"/>
+      <c r="R4" s="29"/>
+      <c r="S4" s="30"/>
       <c r="T4" s="20" t="s">
         <v>28</v>
       </c>
@@ -11657,16 +11657,16 @@
   </sheetData>
   <autoFilter ref="A3:E19" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="10">
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="O4:P4"/>
+    <mergeCell ref="Q4:S4"/>
+    <mergeCell ref="F1:T1"/>
+    <mergeCell ref="U1:V1"/>
     <mergeCell ref="W1:AE1"/>
     <mergeCell ref="F2:M2"/>
     <mergeCell ref="N2:T2"/>
     <mergeCell ref="X2:AA2"/>
     <mergeCell ref="AB2:AE2"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="O4:P4"/>
-    <mergeCell ref="Q4:S4"/>
-    <mergeCell ref="F1:T1"/>
-    <mergeCell ref="U1:V1"/>
   </mergeCells>
   <conditionalFormatting sqref="F5:L19">
     <cfRule type="notContainsBlanks" dxfId="10" priority="2">
@@ -11698,25 +11698,25 @@
       <formula>"Accredited"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="V16">
+    <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
+      <formula>"Accredited"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="W5:W19">
-    <cfRule type="notContainsBlanks" dxfId="4" priority="7">
+    <cfRule type="notContainsBlanks" dxfId="3" priority="7">
       <formula>LEN(TRIM(W5))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X5:AE19">
-    <cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="high">
+    <cfRule type="containsText" dxfId="2" priority="4" operator="containsText" text="high">
       <formula>NOT(ISERROR(SEARCH(("high"),(X5))))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="5" operator="containsText" text="medium">
+    <cfRule type="containsText" dxfId="1" priority="5" operator="containsText" text="medium">
       <formula>NOT(ISERROR(SEARCH(("medium"),(X5))))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="6" operator="containsText" text="low">
+    <cfRule type="containsText" dxfId="0" priority="6" operator="containsText" text="low">
       <formula>NOT(ISERROR(SEARCH(("low"),(X5))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="V16">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
-      <formula>"Accredited"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
sync: partner workbook from Google Drive (2026-06-02 15:04 UTC)
</commit_message>
<xml_diff>
--- a/data/partner/Focus Partner Tracking BR.xlsx
+++ b/data/partner/Focus Partner Tracking BR.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mrovere/Documents/Codex/2026-05-29/acesso-o-google-drive-e-analise/mrovere-treino-push/data/partner/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mrovere/Library/CloudStorage/GoogleDrive-marcelo@mrovere.com/Other computers/My MacBook Pro/Tenable - geral/Internal - Tenable/Canais/2026 news/EM Cert/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8134D0E-2241-0747-815D-CB9C2EC72110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -574,11 +574,14 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -591,14 +594,19 @@
     <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="11">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFCE5CD"/>
+          <bgColor rgb="FFFCE5CD"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -628,14 +636,6 @@
         <patternFill patternType="solid">
           <fgColor rgb="FFC9DAF8"/>
           <bgColor rgb="FFC9DAF8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFCE5CD"/>
-          <bgColor rgb="FFFCE5CD"/>
         </patternFill>
       </fill>
     </dxf>
@@ -945,38 +945,38 @@
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
-      <c r="F1" s="28" t="s">
+      <c r="F1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-      <c r="L1" s="29"/>
-      <c r="M1" s="29"/>
-      <c r="N1" s="29"/>
-      <c r="O1" s="29"/>
-      <c r="P1" s="29"/>
-      <c r="Q1" s="29"/>
-      <c r="R1" s="29"/>
-      <c r="S1" s="29"/>
-      <c r="T1" s="30"/>
-      <c r="U1" s="28" t="s">
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="30"/>
+      <c r="M1" s="30"/>
+      <c r="N1" s="30"/>
+      <c r="O1" s="30"/>
+      <c r="P1" s="30"/>
+      <c r="Q1" s="30"/>
+      <c r="R1" s="30"/>
+      <c r="S1" s="30"/>
+      <c r="T1" s="29"/>
+      <c r="U1" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="V1" s="30"/>
-      <c r="W1" s="28" t="s">
+      <c r="V1" s="29"/>
+      <c r="W1" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="X1" s="29"/>
-      <c r="Y1" s="29"/>
-      <c r="Z1" s="29"/>
-      <c r="AA1" s="29"/>
-      <c r="AB1" s="29"/>
-      <c r="AC1" s="29"/>
-      <c r="AD1" s="29"/>
-      <c r="AE1" s="30"/>
+      <c r="X1" s="30"/>
+      <c r="Y1" s="30"/>
+      <c r="Z1" s="30"/>
+      <c r="AA1" s="30"/>
+      <c r="AB1" s="30"/>
+      <c r="AC1" s="30"/>
+      <c r="AD1" s="30"/>
+      <c r="AE1" s="29"/>
     </row>
     <row r="2" spans="1:31" ht="13" x14ac:dyDescent="0.15">
       <c r="A2" s="2"/>
@@ -984,25 +984,25 @@
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="4"/>
-      <c r="F2" s="31" t="s">
+      <c r="F2" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
-      <c r="J2" s="29"/>
-      <c r="K2" s="29"/>
-      <c r="L2" s="29"/>
-      <c r="M2" s="30"/>
-      <c r="N2" s="32" t="s">
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
+      <c r="K2" s="30"/>
+      <c r="L2" s="30"/>
+      <c r="M2" s="29"/>
+      <c r="N2" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="O2" s="29"/>
-      <c r="P2" s="29"/>
-      <c r="Q2" s="29"/>
-      <c r="R2" s="29"/>
-      <c r="S2" s="29"/>
-      <c r="T2" s="30"/>
+      <c r="O2" s="30"/>
+      <c r="P2" s="30"/>
+      <c r="Q2" s="30"/>
+      <c r="R2" s="30"/>
+      <c r="S2" s="30"/>
+      <c r="T2" s="29"/>
       <c r="U2" s="5" t="s">
         <v>5</v>
       </c>
@@ -1012,18 +1012,18 @@
       <c r="W2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="X2" s="33" t="s">
+      <c r="X2" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="Y2" s="29"/>
-      <c r="Z2" s="29"/>
-      <c r="AA2" s="30"/>
-      <c r="AB2" s="34" t="s">
+      <c r="Y2" s="30"/>
+      <c r="Z2" s="30"/>
+      <c r="AA2" s="29"/>
+      <c r="AB2" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="AC2" s="29"/>
-      <c r="AD2" s="29"/>
-      <c r="AE2" s="30"/>
+      <c r="AC2" s="30"/>
+      <c r="AD2" s="30"/>
+      <c r="AE2" s="29"/>
     </row>
     <row r="3" spans="1:31" ht="13" x14ac:dyDescent="0.15">
       <c r="A3" s="8" t="s">
@@ -1125,10 +1125,10 @@
       <c r="F4" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="G4" s="35" t="s">
+      <c r="G4" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="H4" s="30"/>
+      <c r="H4" s="29"/>
       <c r="I4" s="20" t="s">
         <v>28</v>
       </c>
@@ -1147,15 +1147,15 @@
       <c r="N4" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="O4" s="35" t="s">
+      <c r="O4" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="P4" s="30"/>
-      <c r="Q4" s="35" t="s">
+      <c r="P4" s="29"/>
+      <c r="Q4" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="R4" s="29"/>
-      <c r="S4" s="30"/>
+      <c r="R4" s="30"/>
+      <c r="S4" s="29"/>
       <c r="T4" s="20" t="s">
         <v>28</v>
       </c>
@@ -11657,16 +11657,16 @@
   </sheetData>
   <autoFilter ref="A3:E19" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="10">
+    <mergeCell ref="W1:AE1"/>
+    <mergeCell ref="F2:M2"/>
+    <mergeCell ref="N2:T2"/>
+    <mergeCell ref="X2:AA2"/>
+    <mergeCell ref="AB2:AE2"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="O4:P4"/>
     <mergeCell ref="Q4:S4"/>
     <mergeCell ref="F1:T1"/>
     <mergeCell ref="U1:V1"/>
-    <mergeCell ref="W1:AE1"/>
-    <mergeCell ref="F2:M2"/>
-    <mergeCell ref="N2:T2"/>
-    <mergeCell ref="X2:AA2"/>
-    <mergeCell ref="AB2:AE2"/>
   </mergeCells>
   <conditionalFormatting sqref="F5:L19">
     <cfRule type="notContainsBlanks" dxfId="10" priority="2">
@@ -11698,25 +11698,25 @@
       <formula>"Accredited"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V16">
-    <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
-      <formula>"Accredited"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="W5:W19">
-    <cfRule type="notContainsBlanks" dxfId="3" priority="7">
+    <cfRule type="notContainsBlanks" dxfId="4" priority="7">
       <formula>LEN(TRIM(W5))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X5:AE19">
-    <cfRule type="containsText" dxfId="2" priority="4" operator="containsText" text="high">
+    <cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="high">
       <formula>NOT(ISERROR(SEARCH(("high"),(X5))))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="5" operator="containsText" text="medium">
+    <cfRule type="containsText" dxfId="2" priority="5" operator="containsText" text="medium">
       <formula>NOT(ISERROR(SEARCH(("medium"),(X5))))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="6" operator="containsText" text="low">
+    <cfRule type="containsText" dxfId="1" priority="6" operator="containsText" text="low">
       <formula>NOT(ISERROR(SEARCH(("low"),(X5))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V16">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+      <formula>"Accredited"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: adiciona aba Guardian com 12 candidatos (VM Sales/VM SE/TCDE)
</commit_message>
<xml_diff>
--- a/data/partner/Focus Partner Tracking BR.xlsx
+++ b/data/partner/Focus Partner Tracking BR.xlsx
@@ -3,11 +3,12 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16960" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16960" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="BR" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Tech Certs" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Guardian" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BR'!$A$3:$E$19</definedName>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="11">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -33,11 +34,6 @@
       <color rgb="FFFFFFFF"/>
       <sz val="16"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -68,8 +64,40 @@
       <color theme="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Roboto"/>
+      <color rgb="FF434343"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Roboto"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="12"/>
+      <u val="single"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -148,8 +176,20 @@
         <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF6F8F9"/>
+        <bgColor rgb="FFF6F8F9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="12">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -284,110 +324,187 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFFFFFFF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFFFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFFFFFF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF284E3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFFFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFFFFFF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFF6F8F9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFF6F8F9"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFF6F8F9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFF6F8F9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF284E3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFF6F8F9"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFF6F8F9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFF6F8F9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="15" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="15" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="15" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
-  <dxfs count="11">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFCE5CD"/>
-          <bgColor rgb="FFFCE5CD"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="15">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -417,6 +534,14 @@
         <patternFill patternType="solid">
           <fgColor rgb="FFC9DAF8"/>
           <bgColor rgb="FFC9DAF8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFCE5CD"/>
+          <bgColor rgb="FFFCE5CD"/>
         </patternFill>
       </fill>
     </dxf>
@@ -468,8 +593,55 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF6F8F9"/>
+          <bgColor rgb="FFF6F8F9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF356854"/>
+          <bgColor rgb="FF356854"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF356854"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF356854"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF356854"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF356854"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="Guardian-style" pivot="0" count="4">
+      <tableStyleElement type="wholeTable" size="0" dxfId="14"/>
+      <tableStyleElement type="headerRow" dxfId="13"/>
+      <tableStyleElement type="firstRowStripe" dxfId="12"/>
+      <tableStyleElement type="secondRowStripe" dxfId="11"/>
+    </tableStyle>
+  </tableStyles>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -765,44 +937,44 @@
       <c r="C1" s="1" t="n"/>
       <c r="D1" s="1" t="n"/>
       <c r="E1" s="1" t="n"/>
-      <c r="F1" s="36" t="inlineStr">
+      <c r="F1" s="32" t="inlineStr">
         <is>
           <t>Cursos e certificacoes</t>
         </is>
       </c>
-      <c r="G1" s="37" t="n"/>
-      <c r="H1" s="37" t="n"/>
-      <c r="I1" s="37" t="n"/>
-      <c r="J1" s="37" t="n"/>
-      <c r="K1" s="37" t="n"/>
-      <c r="L1" s="37" t="n"/>
-      <c r="M1" s="37" t="n"/>
-      <c r="N1" s="37" t="n"/>
-      <c r="O1" s="37" t="n"/>
-      <c r="P1" s="37" t="n"/>
-      <c r="Q1" s="37" t="n"/>
-      <c r="R1" s="37" t="n"/>
-      <c r="S1" s="37" t="n"/>
-      <c r="T1" s="38" t="n"/>
-      <c r="U1" s="36" t="inlineStr">
+      <c r="G1" s="31" t="n"/>
+      <c r="H1" s="31" t="n"/>
+      <c r="I1" s="31" t="n"/>
+      <c r="J1" s="31" t="n"/>
+      <c r="K1" s="31" t="n"/>
+      <c r="L1" s="31" t="n"/>
+      <c r="M1" s="31" t="n"/>
+      <c r="N1" s="31" t="n"/>
+      <c r="O1" s="31" t="n"/>
+      <c r="P1" s="31" t="n"/>
+      <c r="Q1" s="31" t="n"/>
+      <c r="R1" s="31" t="n"/>
+      <c r="S1" s="31" t="n"/>
+      <c r="T1" s="29" t="n"/>
+      <c r="U1" s="32" t="inlineStr">
         <is>
           <t>EM Delivery</t>
         </is>
       </c>
-      <c r="V1" s="38" t="n"/>
-      <c r="W1" s="36" t="inlineStr">
+      <c r="V1" s="29" t="n"/>
+      <c r="W1" s="32" t="inlineStr">
         <is>
           <t>Pre Sales Delivery</t>
         </is>
       </c>
-      <c r="X1" s="37" t="n"/>
-      <c r="Y1" s="37" t="n"/>
-      <c r="Z1" s="37" t="n"/>
-      <c r="AA1" s="37" t="n"/>
-      <c r="AB1" s="37" t="n"/>
-      <c r="AC1" s="37" t="n"/>
-      <c r="AD1" s="37" t="n"/>
-      <c r="AE1" s="38" t="n"/>
+      <c r="X1" s="31" t="n"/>
+      <c r="Y1" s="31" t="n"/>
+      <c r="Z1" s="31" t="n"/>
+      <c r="AA1" s="31" t="n"/>
+      <c r="AB1" s="31" t="n"/>
+      <c r="AC1" s="31" t="n"/>
+      <c r="AD1" s="31" t="n"/>
+      <c r="AE1" s="29" t="n"/>
     </row>
     <row r="2" ht="13" customHeight="1">
       <c r="A2" s="2" t="n"/>
@@ -810,29 +982,29 @@
       <c r="C2" s="3" t="n"/>
       <c r="D2" s="3" t="n"/>
       <c r="E2" s="4" t="n"/>
-      <c r="F2" s="12" t="inlineStr">
+      <c r="F2" s="30" t="inlineStr">
         <is>
           <t>Introduction</t>
         </is>
       </c>
-      <c r="G2" s="37" t="n"/>
-      <c r="H2" s="37" t="n"/>
-      <c r="I2" s="37" t="n"/>
-      <c r="J2" s="37" t="n"/>
-      <c r="K2" s="37" t="n"/>
-      <c r="L2" s="37" t="n"/>
-      <c r="M2" s="38" t="n"/>
-      <c r="N2" s="13" t="inlineStr">
+      <c r="G2" s="31" t="n"/>
+      <c r="H2" s="31" t="n"/>
+      <c r="I2" s="31" t="n"/>
+      <c r="J2" s="31" t="n"/>
+      <c r="K2" s="31" t="n"/>
+      <c r="L2" s="31" t="n"/>
+      <c r="M2" s="29" t="n"/>
+      <c r="N2" s="35" t="inlineStr">
         <is>
           <t>Specialist</t>
         </is>
       </c>
-      <c r="O2" s="37" t="n"/>
-      <c r="P2" s="37" t="n"/>
-      <c r="Q2" s="37" t="n"/>
-      <c r="R2" s="37" t="n"/>
-      <c r="S2" s="37" t="n"/>
-      <c r="T2" s="38" t="n"/>
+      <c r="O2" s="31" t="n"/>
+      <c r="P2" s="31" t="n"/>
+      <c r="Q2" s="31" t="n"/>
+      <c r="R2" s="31" t="n"/>
+      <c r="S2" s="31" t="n"/>
+      <c r="T2" s="29" t="n"/>
       <c r="U2" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">EM </t>
@@ -848,22 +1020,22 @@
           <t>Guardian</t>
         </is>
       </c>
-      <c r="X2" s="15" t="inlineStr">
+      <c r="X2" s="33" t="inlineStr">
         <is>
           <t>Demo</t>
         </is>
       </c>
-      <c r="Y2" s="37" t="n"/>
-      <c r="Z2" s="37" t="n"/>
-      <c r="AA2" s="38" t="n"/>
-      <c r="AB2" s="16" t="inlineStr">
+      <c r="Y2" s="31" t="n"/>
+      <c r="Z2" s="31" t="n"/>
+      <c r="AA2" s="29" t="n"/>
+      <c r="AB2" s="34" t="inlineStr">
         <is>
           <t>POV</t>
         </is>
       </c>
-      <c r="AC2" s="37" t="n"/>
-      <c r="AD2" s="37" t="n"/>
-      <c r="AE2" s="38" t="n"/>
+      <c r="AC2" s="31" t="n"/>
+      <c r="AD2" s="31" t="n"/>
+      <c r="AE2" s="29" t="n"/>
     </row>
     <row r="3" ht="13" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
@@ -892,72 +1064,72 @@
           <t>ONE</t>
         </is>
       </c>
-      <c r="G3" s="12" t="inlineStr">
+      <c r="G3" s="30" t="inlineStr">
         <is>
           <t>VM</t>
         </is>
       </c>
-      <c r="H3" s="12" t="inlineStr">
+      <c r="H3" s="30" t="inlineStr">
         <is>
           <t>SC</t>
         </is>
       </c>
-      <c r="I3" s="12" t="inlineStr">
+      <c r="I3" s="30" t="inlineStr">
         <is>
           <t>WAS</t>
         </is>
       </c>
-      <c r="J3" s="12" t="inlineStr">
+      <c r="J3" s="30" t="inlineStr">
         <is>
           <t>IE</t>
         </is>
       </c>
-      <c r="K3" s="12" t="inlineStr">
+      <c r="K3" s="30" t="inlineStr">
         <is>
           <t>OT</t>
         </is>
       </c>
-      <c r="L3" s="12" t="inlineStr">
+      <c r="L3" s="30" t="inlineStr">
         <is>
           <t>CS</t>
         </is>
       </c>
-      <c r="M3" s="12" t="inlineStr">
+      <c r="M3" s="30" t="inlineStr">
         <is>
           <t>Intro CERT</t>
         </is>
       </c>
-      <c r="N3" s="13" t="inlineStr">
+      <c r="N3" s="35" t="inlineStr">
         <is>
           <t>ONE</t>
         </is>
       </c>
-      <c r="O3" s="13" t="inlineStr">
+      <c r="O3" s="35" t="inlineStr">
         <is>
           <t>VM</t>
         </is>
       </c>
-      <c r="P3" s="13" t="inlineStr">
+      <c r="P3" s="35" t="inlineStr">
         <is>
           <t>SC</t>
         </is>
       </c>
-      <c r="Q3" s="13" t="inlineStr">
+      <c r="Q3" s="35" t="inlineStr">
         <is>
           <t>IE</t>
         </is>
       </c>
-      <c r="R3" s="13" t="inlineStr">
+      <c r="R3" s="35" t="inlineStr">
         <is>
           <t>OT</t>
         </is>
       </c>
-      <c r="S3" s="13" t="inlineStr">
+      <c r="S3" s="35" t="inlineStr">
         <is>
           <t>CS</t>
         </is>
       </c>
-      <c r="T3" s="13" t="inlineStr">
+      <c r="T3" s="35" t="inlineStr">
         <is>
           <t>SP CERT</t>
         </is>
@@ -973,42 +1145,42 @@
         </is>
       </c>
       <c r="W3" s="14" t="n"/>
-      <c r="X3" s="15" t="inlineStr">
+      <c r="X3" s="33" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
       </c>
-      <c r="Y3" s="15" t="inlineStr">
+      <c r="Y3" s="33" t="inlineStr">
         <is>
           <t>VM/WAS</t>
         </is>
       </c>
-      <c r="Z3" s="15" t="inlineStr">
+      <c r="Z3" s="33" t="inlineStr">
         <is>
           <t>CS</t>
         </is>
       </c>
-      <c r="AA3" s="15" t="inlineStr">
+      <c r="AA3" s="33" t="inlineStr">
         <is>
           <t>TPM</t>
         </is>
       </c>
-      <c r="AB3" s="16" t="inlineStr">
+      <c r="AB3" s="34" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
       </c>
-      <c r="AC3" s="16" t="inlineStr">
+      <c r="AC3" s="34" t="inlineStr">
         <is>
           <t>VM/WAS</t>
         </is>
       </c>
-      <c r="AD3" s="16" t="inlineStr">
+      <c r="AD3" s="34" t="inlineStr">
         <is>
           <t>CS</t>
         </is>
       </c>
-      <c r="AE3" s="16" t="inlineStr">
+      <c r="AE3" s="34" t="inlineStr">
         <is>
           <t>TPM</t>
         </is>
@@ -1025,12 +1197,12 @@
           <t>Req</t>
         </is>
       </c>
-      <c r="G4" s="39" t="inlineStr">
+      <c r="G4" s="28" t="inlineStr">
         <is>
           <t>1 out of 2</t>
         </is>
       </c>
-      <c r="H4" s="38" t="n"/>
+      <c r="H4" s="29" t="n"/>
       <c r="I4" s="20" t="inlineStr">
         <is>
           <t>Req</t>
@@ -1061,19 +1233,19 @@
           <t>Req</t>
         </is>
       </c>
-      <c r="O4" s="39" t="inlineStr">
+      <c r="O4" s="28" t="inlineStr">
         <is>
           <t>1 out of 2</t>
         </is>
       </c>
-      <c r="P4" s="38" t="n"/>
-      <c r="Q4" s="39" t="inlineStr">
+      <c r="P4" s="29" t="n"/>
+      <c r="Q4" s="28" t="inlineStr">
         <is>
           <t>2 out of 3</t>
         </is>
       </c>
-      <c r="R4" s="37" t="n"/>
-      <c r="S4" s="38" t="n"/>
+      <c r="R4" s="31" t="n"/>
+      <c r="S4" s="29" t="n"/>
       <c r="T4" s="20" t="inlineStr">
         <is>
           <t>Req</t>
@@ -11919,12 +12091,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N5:S19">
-    <cfRule type="notContainsBlanks" priority="3" dxfId="0">
+    <cfRule type="notContainsBlanks" priority="3" dxfId="4">
       <formula>LEN(TRIM(N5))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T5:T19">
-    <cfRule type="cellIs" priority="10" operator="equal" dxfId="0">
+    <cfRule type="cellIs" priority="10" operator="equal" dxfId="4">
       <formula>"Accredited"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11938,25 +12110,25 @@
       <formula>"Accredited"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="V16">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="4">
+      <formula>"Accredited"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="W5:W19">
-    <cfRule type="notContainsBlanks" priority="7" dxfId="4">
+    <cfRule type="notContainsBlanks" priority="7" dxfId="3">
       <formula>LEN(TRIM(W5))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X5:AE19">
-    <cfRule type="containsText" priority="4" operator="containsText" dxfId="3" text="high">
+    <cfRule type="containsText" priority="4" operator="containsText" dxfId="2" text="high">
       <formula>NOT(ISERROR(SEARCH(("high"),(X5))))</formula>
     </cfRule>
-    <cfRule type="containsText" priority="5" operator="containsText" dxfId="2" text="medium">
+    <cfRule type="containsText" priority="5" operator="containsText" dxfId="1" text="medium">
       <formula>NOT(ISERROR(SEARCH(("medium"),(X5))))</formula>
     </cfRule>
-    <cfRule type="containsText" priority="6" operator="containsText" dxfId="1" text="low">
+    <cfRule type="containsText" priority="6" operator="containsText" dxfId="0" text="low">
       <formula>NOT(ISERROR(SEARCH(("low"),(X5))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="V16">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>"Accredited"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11970,617 +12142,1077 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:P13"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ID Reseller</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>VM-SE</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>VM-Sales</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>CS-SE</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>CS-Sales</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>OT-SE</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>OT-Sales</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>IE-SE</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>IE-Sales</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>ASM-SE</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>ASM-Sales</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Nessus</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>ONE-SE</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>ONE-Sales</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>MSSP</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>581437</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Shield</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>28</v>
+      </c>
+      <c r="D2" t="n">
+        <v>30</v>
+      </c>
+      <c r="E2" t="n">
+        <v>12</v>
+      </c>
+      <c r="F2" t="n">
+        <v>30</v>
+      </c>
+      <c r="G2" t="n">
+        <v>17</v>
+      </c>
+      <c r="H2" t="n">
+        <v>49</v>
+      </c>
+      <c r="I2" t="n">
+        <v>12</v>
+      </c>
+      <c r="J2" t="n">
+        <v>38</v>
+      </c>
+      <c r="K2" t="n">
+        <v>12</v>
+      </c>
+      <c r="L2" t="n">
+        <v>37</v>
+      </c>
+      <c r="M2" t="n">
+        <v>40</v>
+      </c>
+      <c r="N2" t="n">
+        <v>21</v>
+      </c>
+      <c r="O2" t="n">
+        <v>64</v>
+      </c>
+      <c r="P2" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>390733</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TDEC</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="n">
+        <v>3</v>
+      </c>
+      <c r="K3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" t="n">
+        <v>1</v>
+      </c>
+      <c r="N3" t="n">
+        <v>1</v>
+      </c>
+      <c r="O3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>739732</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Asper</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J4" t="n">
+        <v>8</v>
+      </c>
+      <c r="K4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M4" t="n">
+        <v>4</v>
+      </c>
+      <c r="N4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>579399</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>XSITE</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>7</v>
+      </c>
+      <c r="D5" t="n">
+        <v>7</v>
+      </c>
+      <c r="E5" t="n">
+        <v>9</v>
+      </c>
+      <c r="F5" t="n">
+        <v>7</v>
+      </c>
+      <c r="G5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" t="n">
+        <v>4</v>
+      </c>
+      <c r="I5" t="n">
+        <v>8</v>
+      </c>
+      <c r="J5" t="n">
+        <v>9</v>
+      </c>
+      <c r="K5" t="n">
+        <v>4</v>
+      </c>
+      <c r="L5" t="n">
+        <v>6</v>
+      </c>
+      <c r="M5" t="n">
+        <v>5</v>
+      </c>
+      <c r="N5" t="n">
+        <v>5</v>
+      </c>
+      <c r="O5" t="n">
+        <v>8</v>
+      </c>
+      <c r="P5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>397166</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ISH</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>14</v>
+      </c>
+      <c r="D6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E6" t="n">
+        <v>7</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H6" t="n">
+        <v>9</v>
+      </c>
+      <c r="I6" t="n">
+        <v>4</v>
+      </c>
+      <c r="J6" t="n">
+        <v>8</v>
+      </c>
+      <c r="K6" t="n">
+        <v>3</v>
+      </c>
+      <c r="L6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M6" t="n">
+        <v>9</v>
+      </c>
+      <c r="N6" t="n">
+        <v>5</v>
+      </c>
+      <c r="O6" t="n">
+        <v>15</v>
+      </c>
+      <c r="P6" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>993857</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>GlobaslSec</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>510201</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>NetSecurity</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" t="n">
+        <v>6</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" t="n">
+        <v>4</v>
+      </c>
+      <c r="M8" t="n">
+        <v>3</v>
+      </c>
+      <c r="N8" t="n">
+        <v>2</v>
+      </c>
+      <c r="O8" t="n">
+        <v>7</v>
+      </c>
+      <c r="P8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>458265</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" t="n">
+        <v>3</v>
+      </c>
+      <c r="H9" t="n">
+        <v>5</v>
+      </c>
+      <c r="I9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J9" t="n">
+        <v>4</v>
+      </c>
+      <c r="K9" t="n">
+        <v>2</v>
+      </c>
+      <c r="L9" t="n">
+        <v>4</v>
+      </c>
+      <c r="M9" t="n">
+        <v>4</v>
+      </c>
+      <c r="N9" t="n">
+        <v>4</v>
+      </c>
+      <c r="O9" t="n">
+        <v>6</v>
+      </c>
+      <c r="P9" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>119472</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Accenture</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" t="n">
+        <v>2</v>
+      </c>
+      <c r="K10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1</v>
+      </c>
+      <c r="O10" t="n">
+        <v>2</v>
+      </c>
+      <c r="P10" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>106294</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Under Protection</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>5</v>
+      </c>
+      <c r="D11" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" t="n">
+        <v>5</v>
+      </c>
+      <c r="F11" t="n">
+        <v>6</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2</v>
+      </c>
+      <c r="H11" t="n">
+        <v>5</v>
+      </c>
+      <c r="I11" t="n">
+        <v>4</v>
+      </c>
+      <c r="J11" t="n">
+        <v>5</v>
+      </c>
+      <c r="K11" t="n">
+        <v>3</v>
+      </c>
+      <c r="L11" t="n">
+        <v>4</v>
+      </c>
+      <c r="M11" t="n">
+        <v>5</v>
+      </c>
+      <c r="N11" t="n">
+        <v>6</v>
+      </c>
+      <c r="O11" t="n">
+        <v>8</v>
+      </c>
+      <c r="P11" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>543439</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Kryptus</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1</v>
+      </c>
+      <c r="O12" t="n">
+        <v>4</v>
+      </c>
+      <c r="P12" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>686107</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>E-Safer</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>5</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>6</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" t="n">
+        <v>4</v>
+      </c>
+      <c r="J13" t="n">
+        <v>5</v>
+      </c>
+      <c r="L13" t="n">
+        <v>4</v>
+      </c>
+      <c r="M13" t="n">
+        <v>4</v>
+      </c>
+      <c r="N13" t="n">
+        <v>3</v>
+      </c>
+      <c r="O13" t="n">
+        <v>9</v>
+      </c>
+      <c r="P13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>ID Reseller</t>
+          <t>Guardian Name</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>Partner</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>VM-SE</t>
-        </is>
-      </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>VM-Sales</t>
+          <t>Specialist Course</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>CS-SE</t>
+          <t>TCSA</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>CS-Sales</t>
+          <t>TCSE</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>OT-SE</t>
+          <t>TCDE</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>OT-Sales</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>IE-SE</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>IE-Sales</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>ASM-SE</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>ASM-Sales</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Nessus</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>ONE-SE</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>ONE-Sales</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>MSSP</t>
+          <t>Obs</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>581437</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Daniel Batista</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>daniel.batista@shieldsec.com.br</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>Shield</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>28</v>
-      </c>
-      <c r="D2" t="n">
-        <v>30</v>
-      </c>
-      <c r="E2" t="n">
-        <v>12</v>
-      </c>
-      <c r="F2" t="n">
-        <v>30</v>
-      </c>
-      <c r="G2" t="n">
-        <v>17</v>
-      </c>
-      <c r="H2" t="n">
-        <v>49</v>
-      </c>
-      <c r="I2" t="n">
-        <v>12</v>
-      </c>
-      <c r="J2" t="n">
-        <v>38</v>
-      </c>
-      <c r="K2" t="n">
-        <v>12</v>
-      </c>
-      <c r="L2" t="n">
-        <v>37</v>
-      </c>
-      <c r="M2" t="n">
-        <v>40</v>
-      </c>
-      <c r="N2" t="n">
-        <v>21</v>
-      </c>
-      <c r="O2" t="n">
-        <v>64</v>
-      </c>
-      <c r="P2" t="n">
-        <v>11</v>
+      <c r="D2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>faltam provas</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>390733</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Enalta Diniz</t>
+        </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>elnata.diniz@shieldsec.com.br</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Shield</t>
+        </is>
+      </c>
+      <c r="D3" t="b">
+        <v>1</v>
+      </c>
+      <c r="E3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" t="b">
+        <v>0</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>faltam provas</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Raul Carbonari</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>rcarbonari@tdec.com.br</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>TDEC</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="D4" t="b">
         <v>1</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E4" t="b">
         <v>1</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F4" t="b">
         <v>1</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G4" t="b">
+        <v>0</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>faltam provas</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>David Celestino</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>david.celestino@asper.tec.br</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Asper</t>
+        </is>
+      </c>
+      <c r="D5" t="b">
         <v>1</v>
       </c>
-      <c r="G3" t="n">
+      <c r="E5" t="b">
         <v>1</v>
       </c>
-      <c r="H3" t="n">
+      <c r="F5" t="b">
         <v>1</v>
       </c>
-      <c r="I3" t="n">
+      <c r="G5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>faltam provas</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Avner Nahum</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>avner.nahum@asper.tec.br</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Asper</t>
+        </is>
+      </c>
+      <c r="D6" t="b">
         <v>1</v>
       </c>
-      <c r="J3" t="n">
-        <v>3</v>
-      </c>
-      <c r="K3" t="n">
+      <c r="E6" t="b">
         <v>1</v>
       </c>
-      <c r="L3" t="n">
+      <c r="F6" t="b">
         <v>1</v>
       </c>
-      <c r="M3" t="n">
+      <c r="G6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>faltam provas</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Lucas Vasconcelos</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>lucas.silva@globalsectec.com.br</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>GlobalSec</t>
+        </is>
+      </c>
+      <c r="D7" t="b">
+        <v>0</v>
+      </c>
+      <c r="E7" t="b">
+        <v>0</v>
+      </c>
+      <c r="F7" t="b">
+        <v>0</v>
+      </c>
+      <c r="G7" t="b">
+        <v>0</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>realizando curso intro para liberar especialista</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ISH</t>
+        </is>
+      </c>
+      <c r="D8" t="b">
+        <v>0</v>
+      </c>
+      <c r="E8" t="b">
+        <v>0</v>
+      </c>
+      <c r="F8" t="b">
+        <v>0</v>
+      </c>
+      <c r="G8" t="b">
+        <v>0</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>aguardando o nelson</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Alessandro Vitalino</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>alessandro.vitalino@netsecurity.com.br</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Netsecurity</t>
+        </is>
+      </c>
+      <c r="D9" t="b">
+        <v>0</v>
+      </c>
+      <c r="E9" t="b">
         <v>1</v>
       </c>
-      <c r="N3" t="n">
+      <c r="F9" t="b">
         <v>1</v>
       </c>
-      <c r="O3" t="n">
+      <c r="G9" t="b">
+        <v>0</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>cursos liberados</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Gutenberg Brito</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>gutenberg.brito@netsecurity.com.br</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Netsecurity</t>
+        </is>
+      </c>
+      <c r="D10" t="b">
+        <v>0</v>
+      </c>
+      <c r="E10" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>739732</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Asper</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D4" t="n">
-        <v>6</v>
-      </c>
-      <c r="E4" t="n">
-        <v>5</v>
-      </c>
-      <c r="F4" t="n">
-        <v>4</v>
-      </c>
-      <c r="G4" t="n">
-        <v>3</v>
-      </c>
-      <c r="H4" t="n">
-        <v>5</v>
-      </c>
-      <c r="I4" t="n">
-        <v>4</v>
-      </c>
-      <c r="J4" t="n">
-        <v>8</v>
-      </c>
-      <c r="K4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L4" t="n">
-        <v>3</v>
-      </c>
-      <c r="M4" t="n">
-        <v>4</v>
-      </c>
-      <c r="N4" t="n">
-        <v>5</v>
-      </c>
-      <c r="O4" t="n">
-        <v>7</v>
-      </c>
-      <c r="P4" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>579399</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>XSITE</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>7</v>
-      </c>
-      <c r="D5" t="n">
-        <v>7</v>
-      </c>
-      <c r="E5" t="n">
-        <v>9</v>
-      </c>
-      <c r="F5" t="n">
-        <v>7</v>
-      </c>
-      <c r="G5" t="n">
-        <v>3</v>
-      </c>
-      <c r="H5" t="n">
-        <v>4</v>
-      </c>
-      <c r="I5" t="n">
-        <v>8</v>
-      </c>
-      <c r="J5" t="n">
-        <v>9</v>
-      </c>
-      <c r="K5" t="n">
-        <v>4</v>
-      </c>
-      <c r="L5" t="n">
-        <v>6</v>
-      </c>
-      <c r="M5" t="n">
-        <v>5</v>
-      </c>
-      <c r="N5" t="n">
-        <v>5</v>
-      </c>
-      <c r="O5" t="n">
-        <v>8</v>
-      </c>
-      <c r="P5" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>397166</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>ISH</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>14</v>
-      </c>
-      <c r="D6" t="n">
-        <v>20</v>
-      </c>
-      <c r="E6" t="n">
-        <v>7</v>
-      </c>
-      <c r="F6" t="n">
-        <v>4</v>
-      </c>
-      <c r="G6" t="n">
-        <v>9</v>
-      </c>
-      <c r="H6" t="n">
-        <v>9</v>
-      </c>
-      <c r="I6" t="n">
-        <v>4</v>
-      </c>
-      <c r="J6" t="n">
-        <v>8</v>
-      </c>
-      <c r="K6" t="n">
-        <v>3</v>
-      </c>
-      <c r="L6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M6" t="n">
-        <v>9</v>
-      </c>
-      <c r="N6" t="n">
-        <v>5</v>
-      </c>
-      <c r="O6" t="n">
-        <v>15</v>
-      </c>
-      <c r="P6" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>993857</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>GlobaslSec</t>
-        </is>
-      </c>
-      <c r="H7" t="n">
+      <c r="F10" t="b">
         <v>1</v>
       </c>
-      <c r="J7" t="n">
+      <c r="G10" t="b">
+        <v>0</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>cursos liberados</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Marco Leissman</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>marco.leissmann@underprotection.com.br</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Underprotection</t>
+        </is>
+      </c>
+      <c r="D11" t="b">
+        <v>0</v>
+      </c>
+      <c r="E11" t="b">
         <v>1</v>
       </c>
-      <c r="N7" t="n">
+      <c r="F11" t="b">
         <v>1</v>
       </c>
-      <c r="O7" t="n">
+      <c r="G11" t="b">
+        <v>0</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>liberar treinamentos. finalizando online</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Ney Gelbcke Junior</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ney.gelbcke@underprotection.com.br</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Underprotection</t>
+        </is>
+      </c>
+      <c r="D12" t="b">
+        <v>0</v>
+      </c>
+      <c r="E12" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>510201</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>NetSecurity</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D8" t="n">
-        <v>6</v>
-      </c>
-      <c r="E8" t="n">
+      <c r="F12" t="b">
         <v>1</v>
       </c>
-      <c r="F8" t="n">
-        <v>4</v>
-      </c>
-      <c r="H8" t="n">
+      <c r="G12" t="b">
+        <v>0</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>liberar treinamentos. finalizando online</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Yueslly Lisboa</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>yueslly.lisboa@xsite.com.br</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>XSite</t>
+        </is>
+      </c>
+      <c r="D13" t="b">
         <v>1</v>
       </c>
-      <c r="J8" t="n">
-        <v>2</v>
-      </c>
-      <c r="K8" t="n">
+      <c r="E13" t="b">
         <v>1</v>
       </c>
-      <c r="L8" t="n">
-        <v>4</v>
-      </c>
-      <c r="M8" t="n">
-        <v>3</v>
-      </c>
-      <c r="N8" t="n">
-        <v>2</v>
-      </c>
-      <c r="O8" t="n">
-        <v>7</v>
-      </c>
-      <c r="P8" t="n">
+      <c r="F13" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>458265</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Future</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>5</v>
-      </c>
-      <c r="D9" t="n">
-        <v>5</v>
-      </c>
-      <c r="E9" t="n">
-        <v>3</v>
-      </c>
-      <c r="F9" t="n">
-        <v>3</v>
-      </c>
-      <c r="G9" t="n">
-        <v>3</v>
-      </c>
-      <c r="H9" t="n">
-        <v>5</v>
-      </c>
-      <c r="I9" t="n">
-        <v>2</v>
-      </c>
-      <c r="J9" t="n">
-        <v>4</v>
-      </c>
-      <c r="K9" t="n">
-        <v>2</v>
-      </c>
-      <c r="L9" t="n">
-        <v>4</v>
-      </c>
-      <c r="M9" t="n">
-        <v>4</v>
-      </c>
-      <c r="N9" t="n">
-        <v>4</v>
-      </c>
-      <c r="O9" t="n">
-        <v>6</v>
-      </c>
-      <c r="P9" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>119472</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Accenture</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
+      <c r="G13" t="b">
         <v>1</v>
       </c>
-      <c r="G10" t="n">
-        <v>2</v>
-      </c>
-      <c r="H10" t="n">
-        <v>2</v>
-      </c>
-      <c r="K10" t="n">
-        <v>1</v>
-      </c>
-      <c r="L10" t="n">
-        <v>1</v>
-      </c>
-      <c r="O10" t="n">
-        <v>2</v>
-      </c>
-      <c r="P10" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>106294</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Under Protection</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>5</v>
-      </c>
-      <c r="D11" t="n">
-        <v>5</v>
-      </c>
-      <c r="E11" t="n">
-        <v>5</v>
-      </c>
-      <c r="F11" t="n">
-        <v>6</v>
-      </c>
-      <c r="G11" t="n">
-        <v>2</v>
-      </c>
-      <c r="H11" t="n">
-        <v>5</v>
-      </c>
-      <c r="I11" t="n">
-        <v>4</v>
-      </c>
-      <c r="J11" t="n">
-        <v>5</v>
-      </c>
-      <c r="K11" t="n">
-        <v>3</v>
-      </c>
-      <c r="L11" t="n">
-        <v>4</v>
-      </c>
-      <c r="M11" t="n">
-        <v>5</v>
-      </c>
-      <c r="N11" t="n">
-        <v>6</v>
-      </c>
-      <c r="O11" t="n">
-        <v>8</v>
-      </c>
-      <c r="P11" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>543439</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Kryptus</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H12" t="n">
-        <v>1</v>
-      </c>
-      <c r="O12" t="n">
-        <v>4</v>
-      </c>
-      <c r="P12" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>686107</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>E-Safer</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" t="n">
-        <v>5</v>
-      </c>
-      <c r="E13" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" t="n">
-        <v>6</v>
-      </c>
-      <c r="G13" t="n">
-        <v>1</v>
-      </c>
-      <c r="H13" t="n">
-        <v>4</v>
-      </c>
-      <c r="J13" t="n">
-        <v>5</v>
-      </c>
-      <c r="L13" t="n">
-        <v>4</v>
-      </c>
-      <c r="M13" t="n">
-        <v>4</v>
-      </c>
-      <c r="N13" t="n">
-        <v>3</v>
-      </c>
-      <c r="O13" t="n">
-        <v>9</v>
-      </c>
-      <c r="P13" t="n">
-        <v>1</v>
-      </c>
+      <c r="H13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: certificações EM atualizadas via Tableau (2026-07-06)
</commit_message>
<xml_diff>
--- a/data/partner/Focus Partner Tracking BR.xlsx
+++ b/data/partner/Focus Partner Tracking BR.xlsx
@@ -1161,69 +1161,63 @@
           <t>Gold</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="G5" s="23" t="inlineStr">
+      <c r="H5" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="H5" s="23" t="inlineStr">
+      <c r="I5" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I5" s="23" t="n"/>
-      <c r="J5" s="23" t="inlineStr">
+      <c r="J5" s="23" t="n"/>
+      <c r="K5" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="K5" s="23" t="inlineStr">
+      <c r="L5" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="L5" s="23" t="inlineStr">
+      <c r="M5" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="M5" s="23" t="inlineStr">
+      <c r="N5" s="23" t="inlineStr">
+        <is>
+          <t>Accredited</t>
+        </is>
+      </c>
+      <c r="O5" s="23" t="n"/>
+      <c r="P5" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="N5" s="23" t="n"/>
-      <c r="O5" s="23" t="inlineStr">
+      <c r="Q5" s="23" t="n"/>
+      <c r="R5" s="23" t="n"/>
+      <c r="S5" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="P5" s="23" t="n"/>
-      <c r="Q5" s="23" t="n"/>
-      <c r="R5" s="23" t="inlineStr">
+      <c r="T5" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="S5" s="23" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="T5" s="23" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="U5" s="23" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
+      <c r="U5" s="23">
+        <f>IF(AND(O5&lt;&gt;"", OR(P5&lt;&gt;"", Q5&lt;&gt;""), OR(AND(R5&lt;&gt;"", S5&lt;&gt;""), AND(S5&lt;&gt;"", T5&lt;&gt;""), AND(R5&lt;&gt;"", T5&lt;&gt;""))), "Accredited", "In Progress")</f>
+        <v/>
       </c>
       <c r="V5" s="24" t="inlineStr">
         <is>
@@ -1301,36 +1295,42 @@
         </is>
       </c>
       <c r="G6" s="23" t="n"/>
-      <c r="H6" s="23" t="inlineStr">
+      <c r="H6" s="23" t="n"/>
+      <c r="I6" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I6" s="23" t="n"/>
       <c r="J6" s="23" t="n"/>
-      <c r="K6" s="23" t="inlineStr">
+      <c r="K6" s="23" t="n"/>
+      <c r="L6" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="L6" s="23" t="n"/>
       <c r="M6" s="23" t="n"/>
-      <c r="N6" s="23" t="n"/>
-      <c r="O6" s="23" t="inlineStr">
+      <c r="N6" s="23">
+        <f>IF(AND(G6&lt;&gt;"", OR(H6&lt;&gt;"", I6&lt;&gt;""), J6&lt;&gt;"", K6&lt;&gt;"", L6&lt;&gt;"", M6&lt;&gt;""), "Accredited", "In Progress")</f>
+        <v/>
+      </c>
+      <c r="O6" s="23" t="n"/>
+      <c r="P6" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="P6" s="23" t="n"/>
       <c r="Q6" s="23" t="n"/>
       <c r="R6" s="23" t="n"/>
-      <c r="S6" s="23" t="inlineStr">
+      <c r="S6" s="23" t="n"/>
+      <c r="T6" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="T6" s="23" t="n"/>
-      <c r="U6" s="23" t="n"/>
+      <c r="U6" s="23">
+        <f>IF(AND(O6&lt;&gt;"", OR(P6&lt;&gt;"", Q6&lt;&gt;""), OR(AND(R6&lt;&gt;"", S6&lt;&gt;""), AND(S6&lt;&gt;"", T6&lt;&gt;""), AND(R6&lt;&gt;"", T6&lt;&gt;""))), "Accredited", "In Progress")</f>
+        <v/>
+      </c>
       <c r="V6" s="26" t="n"/>
       <c r="W6" s="23">
         <f>IF(AND(N6="Accredited", U6="Accredited",V6&lt;&gt;""), "Accredited", "In Progress")</f>
@@ -1406,42 +1406,47 @@
           <t>Silver</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="G7" s="23" t="inlineStr">
+      <c r="H7" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="H7" s="23" t="inlineStr">
+      <c r="I7" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I7" s="23" t="n"/>
       <c r="J7" s="23" t="n"/>
-      <c r="K7" s="23" t="inlineStr">
+      <c r="K7" s="23" t="n"/>
+      <c r="L7" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="L7" s="23" t="n"/>
       <c r="M7" s="23" t="n"/>
-      <c r="N7" s="23" t="n"/>
-      <c r="O7" s="23" t="inlineStr">
+      <c r="N7" s="23">
+        <f>IF(AND(G7&lt;&gt;"", OR(H7&lt;&gt;"", I7&lt;&gt;""), J7&lt;&gt;"", K7&lt;&gt;"", L7&lt;&gt;"", M7&lt;&gt;""), "Accredited", "In Progress")</f>
+        <v/>
+      </c>
+      <c r="O7" s="23" t="n"/>
+      <c r="P7" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="P7" s="23" t="n"/>
       <c r="Q7" s="23" t="n"/>
       <c r="R7" s="23" t="n"/>
       <c r="S7" s="23" t="n"/>
       <c r="T7" s="23" t="n"/>
-      <c r="U7" s="23" t="n"/>
+      <c r="U7" s="23">
+        <f>IF(AND(O7&lt;&gt;"", OR(P7&lt;&gt;"", Q7&lt;&gt;""), OR(AND(R7&lt;&gt;"", S7&lt;&gt;""), AND(S7&lt;&gt;"", T7&lt;&gt;""), AND(R7&lt;&gt;"", T7&lt;&gt;""))), "Accredited", "In Progress")</f>
+        <v/>
+      </c>
       <c r="V7" s="26" t="n"/>
       <c r="W7" s="23">
         <f>IF(AND(N7="Accredited", U7="Accredited",V7&lt;&gt;""), "Accredited", "In Progress")</f>
@@ -1513,62 +1518,60 @@
           <t>Gold</t>
         </is>
       </c>
-      <c r="G8" s="23" t="inlineStr">
+      <c r="G8" s="23" t="n"/>
+      <c r="H8" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="H8" s="23" t="inlineStr">
+      <c r="I8" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I8" s="23" t="n"/>
-      <c r="J8" s="23" t="inlineStr">
+      <c r="J8" s="23" t="n"/>
+      <c r="K8" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="K8" s="23" t="inlineStr">
+      <c r="L8" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="L8" s="23" t="inlineStr">
+      <c r="M8" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="M8" s="23" t="inlineStr">
+      <c r="N8" s="23">
+        <f>IF(AND(G8&lt;&gt;"", OR(H8&lt;&gt;"", I8&lt;&gt;""), J8&lt;&gt;"", K8&lt;&gt;"", L8&lt;&gt;"", M8&lt;&gt;""), "Accredited", "In Progress")</f>
+        <v/>
+      </c>
+      <c r="O8" s="23" t="n"/>
+      <c r="P8" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="N8" s="23" t="n"/>
-      <c r="O8" s="23" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="P8" s="23" t="n"/>
       <c r="Q8" s="23" t="n"/>
       <c r="R8" s="23" t="n"/>
-      <c r="S8" s="23" t="inlineStr">
+      <c r="S8" s="23" t="n"/>
+      <c r="T8" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="T8" s="23" t="inlineStr">
+      <c r="U8" s="23">
+        <f>IF(AND(O8&lt;&gt;"", OR(P8&lt;&gt;"", Q8&lt;&gt;""), OR(AND(R8&lt;&gt;"", S8&lt;&gt;""), AND(S8&lt;&gt;"", T8&lt;&gt;""), AND(R8&lt;&gt;"", T8&lt;&gt;""))), "Accredited", "In Progress")</f>
+        <v/>
+      </c>
+      <c r="V8" s="26" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="U8" s="23" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="V8" s="26" t="n"/>
       <c r="W8" s="23">
         <f>IF(AND(N8="Accredited", U8="Accredited",V8&lt;&gt;""), "Accredited", "In Progress")</f>
         <v/>
@@ -1643,65 +1646,58 @@
           <t>Platinum</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="G9" s="23" t="inlineStr">
+      <c r="H9" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="H9" s="23" t="inlineStr">
+      <c r="I9" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I9" s="23" t="n"/>
-      <c r="J9" s="23" t="inlineStr">
+      <c r="J9" s="23" t="n"/>
+      <c r="K9" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="K9" s="23" t="inlineStr">
+      <c r="L9" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="L9" s="23" t="inlineStr">
+      <c r="M9" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="M9" s="23" t="inlineStr">
+      <c r="N9" s="23">
+        <f>IF(AND(G9&lt;&gt;"", OR(H9&lt;&gt;"", I9&lt;&gt;""), J9&lt;&gt;"", K9&lt;&gt;"", L9&lt;&gt;"", M9&lt;&gt;""), "Accredited", "In Progress")</f>
+        <v/>
+      </c>
+      <c r="O9" s="23" t="n"/>
+      <c r="P9" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="N9" s="23" t="n"/>
-      <c r="O9" s="23" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="P9" s="23" t="n"/>
       <c r="Q9" s="23" t="n"/>
       <c r="R9" s="23" t="n"/>
-      <c r="S9" s="23" t="inlineStr">
+      <c r="S9" s="23" t="n"/>
+      <c r="T9" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="T9" s="23" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="U9" s="23" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
+      <c r="U9" s="23">
+        <f>IF(AND(O9&lt;&gt;"", OR(P9&lt;&gt;"", Q9&lt;&gt;""), OR(AND(R9&lt;&gt;"", S9&lt;&gt;""), AND(S9&lt;&gt;"", T9&lt;&gt;""), AND(R9&lt;&gt;"", T9&lt;&gt;""))), "Accredited", "In Progress")</f>
+        <v/>
       </c>
       <c r="V9" s="24" t="inlineStr">
         <is>
@@ -1786,21 +1782,27 @@
       <c r="H10" s="23" t="n"/>
       <c r="I10" s="23" t="n"/>
       <c r="J10" s="23" t="n"/>
-      <c r="K10" s="23" t="inlineStr">
+      <c r="K10" s="23" t="n"/>
+      <c r="L10" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="L10" s="23" t="n"/>
       <c r="M10" s="23" t="n"/>
-      <c r="N10" s="23" t="n"/>
+      <c r="N10" s="23">
+        <f>IF(AND(G10&lt;&gt;"", OR(H10&lt;&gt;"", I10&lt;&gt;""), J10&lt;&gt;"", K10&lt;&gt;"", L10&lt;&gt;"", M10&lt;&gt;""), "Accredited", "In Progress")</f>
+        <v/>
+      </c>
       <c r="O10" s="23" t="n"/>
       <c r="P10" s="23" t="n"/>
       <c r="Q10" s="23" t="n"/>
       <c r="R10" s="23" t="n"/>
       <c r="S10" s="23" t="n"/>
       <c r="T10" s="23" t="n"/>
-      <c r="U10" s="23" t="n"/>
+      <c r="U10" s="23">
+        <f>IF(AND(O10&lt;&gt;"", OR(P10&lt;&gt;"", Q10&lt;&gt;""), OR(AND(R10&lt;&gt;"", S10&lt;&gt;""), AND(S10&lt;&gt;"", T10&lt;&gt;""), AND(R10&lt;&gt;"", T10&lt;&gt;""))), "Accredited", "In Progress")</f>
+        <v/>
+      </c>
       <c r="V10" s="26" t="n"/>
       <c r="W10" s="23">
         <f>IF(AND(N10="Accredited", U10="Accredited",V10&lt;&gt;""), "Accredited", "In Progress")</f>
@@ -1840,59 +1842,60 @@
           <t>Gold</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="G11" s="23" t="inlineStr">
+      <c r="H11" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="H11" s="23" t="inlineStr">
+      <c r="I11" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I11" s="23" t="n"/>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="23" t="n"/>
+      <c r="K11" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="K11" s="23" t="inlineStr">
+      <c r="L11" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="L11" s="23" t="inlineStr">
+      <c r="M11" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="M11" s="23" t="inlineStr">
+      <c r="N11" s="23">
+        <f>IF(AND(G11&lt;&gt;"", OR(H11&lt;&gt;"", I11&lt;&gt;""), J11&lt;&gt;"", K11&lt;&gt;"", L11&lt;&gt;"", M11&lt;&gt;""), "Accredited", "In Progress")</f>
+        <v/>
+      </c>
+      <c r="O11" s="23" t="n"/>
+      <c r="P11" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="N11" s="23" t="n"/>
-      <c r="O11" s="23" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="P11" s="23" t="n"/>
       <c r="Q11" s="23" t="n"/>
       <c r="R11" s="23" t="n"/>
       <c r="S11" s="23" t="n"/>
       <c r="T11" s="23" t="n"/>
-      <c r="U11" s="23" t="inlineStr">
+      <c r="U11" s="23">
+        <f>IF(AND(O11&lt;&gt;"", OR(P11&lt;&gt;"", Q11&lt;&gt;""), OR(AND(R11&lt;&gt;"", S11&lt;&gt;""), AND(S11&lt;&gt;"", T11&lt;&gt;""), AND(R11&lt;&gt;"", T11&lt;&gt;""))), "Accredited", "In Progress")</f>
+        <v/>
+      </c>
+      <c r="V11" s="26" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="V11" s="26" t="n"/>
       <c r="W11" s="23">
         <f>IF(AND(N11="Accredited", U11="Accredited",V11&lt;&gt;""), "Accredited", "In Progress")</f>
         <v/>
@@ -1963,37 +1966,43 @@
           <t>Silver</t>
         </is>
       </c>
-      <c r="G12" s="23" t="inlineStr">
+      <c r="G12" s="23" t="n"/>
+      <c r="H12" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="H12" s="23" t="inlineStr">
+      <c r="I12" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I12" s="23" t="n"/>
       <c r="J12" s="23" t="n"/>
-      <c r="K12" s="23" t="inlineStr">
+      <c r="K12" s="23" t="n"/>
+      <c r="L12" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="L12" s="23" t="n"/>
       <c r="M12" s="23" t="n"/>
-      <c r="N12" s="23" t="n"/>
-      <c r="O12" s="23" t="inlineStr">
+      <c r="N12" s="23">
+        <f>IF(AND(G12&lt;&gt;"", OR(H12&lt;&gt;"", I12&lt;&gt;""), J12&lt;&gt;"", K12&lt;&gt;"", L12&lt;&gt;"", M12&lt;&gt;""), "Accredited", "In Progress")</f>
+        <v/>
+      </c>
+      <c r="O12" s="23" t="n"/>
+      <c r="P12" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="P12" s="23" t="n"/>
       <c r="Q12" s="23" t="n"/>
       <c r="R12" s="23" t="n"/>
       <c r="S12" s="23" t="n"/>
       <c r="T12" s="23" t="n"/>
-      <c r="U12" s="23" t="n"/>
+      <c r="U12" s="23">
+        <f>IF(AND(O12&lt;&gt;"", OR(P12&lt;&gt;"", Q12&lt;&gt;""), OR(AND(R12&lt;&gt;"", S12&lt;&gt;""), AND(S12&lt;&gt;"", T12&lt;&gt;""), AND(R12&lt;&gt;"", T12&lt;&gt;""))), "Accredited", "In Progress")</f>
+        <v/>
+      </c>
       <c r="V12" s="26" t="n"/>
       <c r="W12" s="23">
         <f>IF(AND(N12="Accredited", U12="Accredited",V12&lt;&gt;""), "Accredited", "In Progress")</f>
@@ -2033,44 +2042,42 @@
           <t>Gold</t>
         </is>
       </c>
-      <c r="G13" s="23" t="inlineStr">
+      <c r="G13" s="23" t="n"/>
+      <c r="H13" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="H13" s="23" t="n"/>
       <c r="I13" s="23" t="n"/>
       <c r="J13" s="23" t="n"/>
-      <c r="K13" s="23" t="inlineStr">
+      <c r="K13" s="23" t="n"/>
+      <c r="L13" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="L13" s="23" t="inlineStr">
+      <c r="M13" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="M13" s="23" t="inlineStr">
+      <c r="N13" s="23">
+        <f>IF(AND(G13&lt;&gt;"", OR(H13&lt;&gt;"", I13&lt;&gt;""), J13&lt;&gt;"", K13&lt;&gt;"", L13&lt;&gt;"", M13&lt;&gt;""), "Accredited", "In Progress")</f>
+        <v/>
+      </c>
+      <c r="O13" s="23" t="n"/>
+      <c r="P13" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="N13" s="23" t="n"/>
-      <c r="O13" s="23" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="P13" s="23" t="n"/>
       <c r="Q13" s="23" t="n"/>
       <c r="R13" s="23" t="n"/>
       <c r="S13" s="23" t="n"/>
       <c r="T13" s="23" t="n"/>
-      <c r="U13" s="23" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
+      <c r="U13" s="23">
+        <f>IF(AND(O13&lt;&gt;"", OR(P13&lt;&gt;"", Q13&lt;&gt;""), OR(AND(R13&lt;&gt;"", S13&lt;&gt;""), AND(S13&lt;&gt;"", T13&lt;&gt;""), AND(R13&lt;&gt;"", T13&lt;&gt;""))), "Accredited", "In Progress")</f>
+        <v/>
       </c>
       <c r="V13" s="26" t="inlineStr">
         <is>
@@ -2115,53 +2122,51 @@
           <t>Gold</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="G14" s="23" t="inlineStr">
+      <c r="H14" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="H14" s="23" t="inlineStr">
+      <c r="I14" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I14" s="23" t="n"/>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="23" t="n"/>
+      <c r="K14" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="K14" s="23" t="inlineStr">
+      <c r="L14" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="L14" s="23" t="inlineStr">
+      <c r="M14" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="M14" s="23" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="N14" s="23" t="n"/>
+      <c r="N14" s="23" t="inlineStr">
+        <is>
+          <t>Accredited</t>
+        </is>
+      </c>
       <c r="O14" s="23" t="n"/>
       <c r="P14" s="23" t="n"/>
       <c r="Q14" s="23" t="n"/>
       <c r="R14" s="23" t="n"/>
       <c r="S14" s="23" t="n"/>
       <c r="T14" s="23" t="n"/>
-      <c r="U14" s="23" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
+      <c r="U14" s="23">
+        <f>IF(AND(O14&lt;&gt;"", OR(P14&lt;&gt;"", Q14&lt;&gt;""), OR(AND(R14&lt;&gt;"", S14&lt;&gt;""), AND(S14&lt;&gt;"", T14&lt;&gt;""), AND(R14&lt;&gt;"", T14&lt;&gt;""))), "Accredited", "In Progress")</f>
+        <v/>
       </c>
       <c r="V14" s="24" t="inlineStr">
         <is>
@@ -2238,37 +2243,39 @@
           <t>Bronze</t>
         </is>
       </c>
-      <c r="G15" s="23" t="inlineStr">
+      <c r="G15" s="23" t="n"/>
+      <c r="H15" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="H15" s="23" t="n"/>
       <c r="I15" s="23" t="n"/>
       <c r="J15" s="23" t="n"/>
       <c r="K15" s="23" t="n"/>
-      <c r="L15" s="23" t="inlineStr">
+      <c r="L15" s="23" t="n"/>
+      <c r="M15" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="M15" s="23" t="inlineStr">
+      <c r="N15" s="23">
+        <f>IF(AND(G15&lt;&gt;"", OR(H15&lt;&gt;"", I15&lt;&gt;""), J15&lt;&gt;"", K15&lt;&gt;"", L15&lt;&gt;"", M15&lt;&gt;""), "Accredited", "In Progress")</f>
+        <v/>
+      </c>
+      <c r="O15" s="23" t="n"/>
+      <c r="P15" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="N15" s="23" t="n"/>
-      <c r="O15" s="23" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="P15" s="23" t="n"/>
       <c r="Q15" s="23" t="n"/>
       <c r="R15" s="23" t="n"/>
       <c r="S15" s="23" t="n"/>
       <c r="T15" s="23" t="n"/>
-      <c r="U15" s="23" t="n"/>
+      <c r="U15" s="23">
+        <f>IF(AND(O15&lt;&gt;"", OR(P15&lt;&gt;"", Q15&lt;&gt;""), OR(AND(R15&lt;&gt;"", S15&lt;&gt;""), AND(S15&lt;&gt;"", T15&lt;&gt;""), AND(R15&lt;&gt;"", T15&lt;&gt;""))), "Accredited", "In Progress")</f>
+        <v/>
+      </c>
       <c r="V15" s="23" t="n"/>
       <c r="W15" s="23" t="inlineStr">
         <is>
@@ -2309,37 +2316,39 @@
           <t>Bronze</t>
         </is>
       </c>
-      <c r="G16" s="23" t="inlineStr">
+      <c r="G16" s="23" t="n"/>
+      <c r="H16" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="H16" s="23" t="n"/>
       <c r="I16" s="23" t="n"/>
       <c r="J16" s="23" t="n"/>
-      <c r="K16" s="23" t="inlineStr">
+      <c r="K16" s="23" t="n"/>
+      <c r="L16" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="L16" s="23" t="inlineStr">
+      <c r="M16" s="23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="M16" s="23" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="N16" s="23" t="n"/>
+      <c r="N16" s="23">
+        <f>IF(AND(G16&lt;&gt;"", OR(H16&lt;&gt;"", I16&lt;&gt;""), J16&lt;&gt;"", K16&lt;&gt;"", L16&lt;&gt;"", M16&lt;&gt;""), "Accredited", "In Progress")</f>
+        <v/>
+      </c>
       <c r="O16" s="23" t="n"/>
       <c r="P16" s="23" t="n"/>
       <c r="Q16" s="23" t="n"/>
       <c r="R16" s="23" t="n"/>
       <c r="S16" s="23" t="n"/>
       <c r="T16" s="23" t="n"/>
-      <c r="U16" s="23" t="n"/>
+      <c r="U16" s="23">
+        <f>IF(AND(O16&lt;&gt;"", OR(P16&lt;&gt;"", Q16&lt;&gt;""), OR(AND(R16&lt;&gt;"", S16&lt;&gt;""), AND(S16&lt;&gt;"", T16&lt;&gt;""), AND(R16&lt;&gt;"", T16&lt;&gt;""))), "Accredited", "In Progress")</f>
+        <v/>
+      </c>
       <c r="V16" s="23" t="n"/>
       <c r="W16" s="23">
         <f>IF(AND(Q16&lt;&gt;"", OR(R16&lt;&gt;"", S16&lt;&gt;""), OR(AND(T16&lt;&gt;"", U16&lt;&gt;""), AND(U16&lt;&gt;"", V16&lt;&gt;""), AND(T16&lt;&gt;"", V16&lt;&gt;""))), "Accredited", "In Progress")</f>

</xml_diff>

<commit_message>
Partner dashboard: coluna Partner com wrap + Guardians concluídos (Omar/TDEC, Thiago/ISH)
- Overview e EM Certs: célula do nome do parceiro estreitada (130px) com
  quebra de linha, liberando espaço para as colunas de certificação
- Workbook: aba Guardian com Omar Fernandes (TDEC) e Thiago Gonçalves (ISH)
  como Guardian concluído

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/partner/Focus Partner Tracking BR.xlsx
+++ b/data/partner/Focus Partner Tracking BR.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16960" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BR" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guardian" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tech Certs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="BR" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Guardian" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Tech Certs" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BR'!$A$3:$F$19</definedName>
@@ -5460,7 +5460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="8.6640625" customWidth="1" min="1" max="26"/>
@@ -5611,48 +5611,48 @@
       </c>
     </row>
     <row r="5" ht="13" customHeight="1">
-      <c r="A5" s="27" t="inlineStr">
-        <is>
-          <t>David Celestino</t>
-        </is>
-      </c>
-      <c r="B5" s="27" t="inlineStr">
-        <is>
-          <t>david.celestino@asper.tec.br</t>
-        </is>
-      </c>
-      <c r="C5" s="27" t="inlineStr">
-        <is>
-          <t>Asper</t>
-        </is>
-      </c>
-      <c r="D5" s="27" t="b">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Omar Fernandes</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ocavalcante@tdec.com.br</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TDEC</t>
+        </is>
+      </c>
+      <c r="D5" t="b">
         <v>1</v>
       </c>
-      <c r="E5" s="27" t="b">
+      <c r="E5" t="b">
         <v>1</v>
       </c>
-      <c r="F5" s="27" t="b">
+      <c r="F5" t="b">
         <v>1</v>
       </c>
-      <c r="G5" s="27" t="b">
-        <v>0</v>
-      </c>
-      <c r="H5" s="27" t="inlineStr">
-        <is>
-          <t>faltam provas</t>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Guardian concluído ✅</t>
         </is>
       </c>
     </row>
     <row r="6" ht="13" customHeight="1">
       <c r="A6" s="27" t="inlineStr">
         <is>
-          <t>Avner Nahum</t>
+          <t>David Celestino</t>
         </is>
       </c>
       <c r="B6" s="27" t="inlineStr">
         <is>
-          <t>avner.nahum@asper.tec.br</t>
+          <t>david.celestino@asper.tec.br</t>
         </is>
       </c>
       <c r="C6" s="27" t="inlineStr">
@@ -5681,51 +5681,51 @@
     <row r="7" ht="13" customHeight="1">
       <c r="A7" s="27" t="inlineStr">
         <is>
-          <t>Lucas Vasconcelos</t>
+          <t>Avner Nahum</t>
         </is>
       </c>
       <c r="B7" s="27" t="inlineStr">
         <is>
-          <t>lucas.silva@globalsectec.com.br</t>
+          <t>avner.nahum@asper.tec.br</t>
         </is>
       </c>
       <c r="C7" s="27" t="inlineStr">
         <is>
-          <t>GlobalSec</t>
+          <t>Asper</t>
         </is>
       </c>
       <c r="D7" s="27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7" s="27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F7" s="27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" s="27" t="b">
         <v>0</v>
       </c>
       <c r="H7" s="27" t="inlineStr">
         <is>
-          <t>realizando curso intro para liberar especialista</t>
+          <t>faltam provas</t>
         </is>
       </c>
     </row>
     <row r="8" ht="13" customHeight="1">
       <c r="A8" s="27" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Lucas Vasconcelos</t>
         </is>
       </c>
       <c r="B8" s="27" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>lucas.silva@globalsectec.com.br</t>
         </is>
       </c>
       <c r="C8" s="27" t="inlineStr">
         <is>
-          <t>ISH</t>
+          <t>GlobalSec</t>
         </is>
       </c>
       <c r="D8" s="27" t="b">
@@ -5742,28 +5742,24 @@
       </c>
       <c r="H8" s="27" t="inlineStr">
         <is>
-          <t>aguardando o nelson</t>
+          <t>realizando curso intro para liberar especialista</t>
         </is>
       </c>
     </row>
     <row r="9" ht="13" customHeight="1">
       <c r="A9" s="27" t="inlineStr">
         <is>
-          <t>Alessandro Vitalino</t>
-        </is>
-      </c>
-      <c r="B9" s="27" t="inlineStr">
-        <is>
-          <t>alessandro.vitalino@netsecurity.com.br</t>
-        </is>
-      </c>
+          <t>Thiago Gonçalves</t>
+        </is>
+      </c>
+      <c r="B9" s="27" t="inlineStr"/>
       <c r="C9" s="27" t="inlineStr">
         <is>
-          <t>Netsecurity</t>
+          <t>ISH</t>
         </is>
       </c>
       <c r="D9" s="27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" s="27" t="b">
         <v>1</v>
@@ -5772,23 +5768,23 @@
         <v>1</v>
       </c>
       <c r="G9" s="27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H9" s="27" t="inlineStr">
         <is>
-          <t>cursos liberados</t>
+          <t>Guardian concluído ✅</t>
         </is>
       </c>
     </row>
     <row r="10" ht="13" customHeight="1">
       <c r="A10" s="27" t="inlineStr">
         <is>
-          <t>Gutenberg Brito</t>
+          <t>Alessandro Vitalino</t>
         </is>
       </c>
       <c r="B10" s="27" t="inlineStr">
         <is>
-          <t>gutenberg.brito@netsecurity.com.br</t>
+          <t>alessandro.vitalino@netsecurity.com.br</t>
         </is>
       </c>
       <c r="C10" s="27" t="inlineStr">
@@ -5817,17 +5813,17 @@
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="27" t="inlineStr">
         <is>
-          <t>Marco Leissman</t>
+          <t>Gutenberg Brito</t>
         </is>
       </c>
       <c r="B11" s="27" t="inlineStr">
         <is>
-          <t>marco.leissmann@underprotection.com.br</t>
+          <t>gutenberg.brito@netsecurity.com.br</t>
         </is>
       </c>
       <c r="C11" s="27" t="inlineStr">
         <is>
-          <t>Underprotection</t>
+          <t>Netsecurity</t>
         </is>
       </c>
       <c r="D11" s="27" t="b">
@@ -5844,19 +5840,19 @@
       </c>
       <c r="H11" s="27" t="inlineStr">
         <is>
-          <t>liberar treinamentos. finalizando online</t>
+          <t>cursos liberados</t>
         </is>
       </c>
     </row>
     <row r="12" ht="13" customHeight="1">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>Ney Gelbcke Junior</t>
+          <t>Marco Leissman</t>
         </is>
       </c>
       <c r="B12" s="27" t="inlineStr">
         <is>
-          <t>ney.gelbcke@underprotection.com.br</t>
+          <t>marco.leissmann@underprotection.com.br</t>
         </is>
       </c>
       <c r="C12" s="27" t="inlineStr">
@@ -5885,21 +5881,21 @@
     <row r="13" ht="13" customHeight="1">
       <c r="A13" s="27" t="inlineStr">
         <is>
-          <t>Yueslly Lisboa</t>
+          <t>Ney Gelbcke Junior</t>
         </is>
       </c>
       <c r="B13" s="27" t="inlineStr">
         <is>
-          <t>yueslly.lisboa@xsite.com.br</t>
+          <t>ney.gelbcke@underprotection.com.br</t>
         </is>
       </c>
       <c r="C13" s="27" t="inlineStr">
         <is>
-          <t>XSite</t>
+          <t>Underprotection</t>
         </is>
       </c>
       <c r="D13" s="27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" s="27" t="b">
         <v>1</v>
@@ -5908,6 +5904,40 @@
         <v>1</v>
       </c>
       <c r="G13" s="27" t="b">
+        <v>0</v>
+      </c>
+      <c r="H13" s="27" t="inlineStr">
+        <is>
+          <t>liberar treinamentos. finalizando online</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="27" t="inlineStr">
+        <is>
+          <t>Yueslly Lisboa</t>
+        </is>
+      </c>
+      <c r="B14" s="27" t="inlineStr">
+        <is>
+          <t>yueslly.lisboa@xsite.com.br</t>
+        </is>
+      </c>
+      <c r="C14" s="27" t="inlineStr">
+        <is>
+          <t>XSite</t>
+        </is>
+      </c>
+      <c r="D14" s="27" t="b">
+        <v>1</v>
+      </c>
+      <c r="E14" s="27" t="b">
+        <v>1</v>
+      </c>
+      <c r="F14" s="27" t="b">
+        <v>1</v>
+      </c>
+      <c r="G14" s="27" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Guardian ISH: corrige nome completo e e-mail (Thiago Pereira Gonçalves)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/partner/Focus Partner Tracking BR.xlsx
+++ b/data/partner/Focus Partner Tracking BR.xlsx
@@ -5749,10 +5749,14 @@
     <row r="9" ht="13" customHeight="1">
       <c r="A9" s="27" t="inlineStr">
         <is>
-          <t>Thiago Gonçalves</t>
-        </is>
-      </c>
-      <c r="B9" s="27" t="inlineStr"/>
+          <t>Thiago Pereira Gonçalves</t>
+        </is>
+      </c>
+      <c r="B9" s="27" t="inlineStr">
+        <is>
+          <t>thiago.pereira@ish.com.br</t>
+        </is>
+      </c>
       <c r="C9" s="27" t="inlineStr">
         <is>
           <t>ISH</t>

</xml_diff>

<commit_message>
Fix colunas Tier/Contact no partner dashboard + Yueslly Guardian concluída
- partner-excel.js: Tier mostrava o contato e Contact o nome curto do
  parceiro — corrigido para primaryContact=row[3] (Primary Contact) e
  status=row[4] (Status), conforme layout da aba BR
- Workbook: Yueslly Lisboa (XSite) marcada como Guardian concluído

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/partner/Focus Partner Tracking BR.xlsx
+++ b/data/partner/Focus Partner Tracking BR.xlsx
@@ -5943,6 +5943,11 @@
       </c>
       <c r="G14" s="27" t="b">
         <v>1</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Guardian concluído ✅</t>
+        </is>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
chore: certificações EM atualizadas via Tableau (2026-07-21)
</commit_message>
<xml_diff>
--- a/data/partner/Focus Partner Tracking BR.xlsx
+++ b/data/partner/Focus Partner Tracking BR.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16960" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="BR" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Guardian" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Tech Certs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BR" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guardian" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tech Certs" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BR'!$A$3:$F$19</definedName>
@@ -1318,19 +1318,11 @@
         <v/>
       </c>
       <c r="O6" s="23" t="n"/>
-      <c r="P6" s="23" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="P6" s="23" t="n"/>
       <c r="Q6" s="23" t="n"/>
       <c r="R6" s="23" t="n"/>
       <c r="S6" s="23" t="n"/>
-      <c r="T6" s="23" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="T6" s="23" t="n"/>
       <c r="U6" s="23">
         <f>IF(AND(O6&lt;&gt;"", OR(P6&lt;&gt;"", Q6&lt;&gt;""), OR(AND(R6&lt;&gt;"", S6&lt;&gt;""), AND(S6&lt;&gt;"", T6&lt;&gt;""), AND(R6&lt;&gt;"", T6&lt;&gt;""))), "Accredited", "In Progress")</f>
         <v/>
@@ -1438,11 +1430,7 @@
         <v/>
       </c>
       <c r="O7" s="23" t="n"/>
-      <c r="P7" s="23" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="P7" s="23" t="n"/>
       <c r="Q7" s="23" t="n"/>
       <c r="R7" s="23" t="n"/>
       <c r="S7" s="23" t="n"/>
@@ -7037,19 +7025,19 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D2" t="n">
         <v>21</v>
       </c>
       <c r="E2" t="n">
+        <v>12</v>
+      </c>
+      <c r="F2" t="n">
+        <v>19</v>
+      </c>
+      <c r="G2" t="n">
         <v>11</v>
-      </c>
-      <c r="F2" t="n">
-        <v>20</v>
-      </c>
-      <c r="G2" t="n">
-        <v>12</v>
       </c>
       <c r="H2" t="n">
         <v>35</v>
@@ -7058,13 +7046,13 @@
         <v>12</v>
       </c>
       <c r="J2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="K2" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="L2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="M2" t="n">
         <v>28</v>
@@ -7076,7 +7064,7 @@
         <v>49</v>
       </c>
       <c r="P2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
@@ -7159,7 +7147,7 @@
         <v>5</v>
       </c>
       <c r="J4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K4" t="n">
         <v>2</v>
@@ -7171,7 +7159,7 @@
         <v>4</v>
       </c>
       <c r="N4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O4" t="n">
         <v>7</v>
@@ -7242,13 +7230,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D6" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F6" t="n">
         <v>3</v>
@@ -7272,7 +7260,7 @@
         <v>5</v>
       </c>
       <c r="M6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N6" t="n">
         <v>5</v>
@@ -7293,17 +7281,23 @@
           <t>GLOBAL SEC. TECNOLOGIA &amp; INFORMACAO EIRELI</t>
         </is>
       </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
       <c r="H7" t="n">
         <v>1</v>
       </c>
       <c r="J7" t="n">
         <v>1</v>
       </c>
+      <c r="M7" t="n">
+        <v>1</v>
+      </c>
       <c r="N7" t="n">
         <v>1</v>
       </c>
       <c r="O7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -7365,10 +7359,10 @@
         <v>5</v>
       </c>
       <c r="D9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F9" t="n">
         <v>3</v>
@@ -7377,7 +7371,7 @@
         <v>3</v>
       </c>
       <c r="H9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I9" t="n">
         <v>2</v>
@@ -7389,10 +7383,10 @@
         <v>2</v>
       </c>
       <c r="L9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N9" t="n">
         <v>4</v>
@@ -7401,7 +7395,7 @@
         <v>6</v>
       </c>
       <c r="P9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -7417,10 +7411,10 @@
         <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K10" t="n">
         <v>1</v>
@@ -7445,46 +7439,46 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E11" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F11" t="n">
         <v>5</v>
       </c>
       <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="n">
         <v>2</v>
       </c>
-      <c r="H11" t="n">
+      <c r="I11" t="n">
+        <v>3</v>
+      </c>
+      <c r="J11" t="n">
         <v>4</v>
       </c>
-      <c r="I11" t="n">
+      <c r="K11" t="n">
+        <v>2</v>
+      </c>
+      <c r="L11" t="n">
+        <v>3</v>
+      </c>
+      <c r="M11" t="n">
         <v>4</v>
       </c>
-      <c r="J11" t="n">
+      <c r="N11" t="n">
         <v>5</v>
       </c>
-      <c r="K11" t="n">
-        <v>3</v>
-      </c>
-      <c r="L11" t="n">
-        <v>4</v>
-      </c>
-      <c r="M11" t="n">
-        <v>5</v>
-      </c>
-      <c r="N11" t="n">
+      <c r="O11" t="n">
         <v>6</v>
       </c>
-      <c r="O11" t="n">
-        <v>8</v>
-      </c>
       <c r="P11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
chore: certificações EM atualizadas via Tableau (2026-07-23)
</commit_message>
<xml_diff>
--- a/data/partner/Focus Partner Tracking BR.xlsx
+++ b/data/partner/Focus Partner Tracking BR.xlsx
@@ -1298,7 +1298,11 @@
           <t>Gold</t>
         </is>
       </c>
-      <c r="G6" s="23" t="n"/>
+      <c r="G6" s="23" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="H6" s="23" t="n"/>
       <c r="I6" s="23" t="inlineStr">
         <is>
@@ -1318,16 +1322,28 @@
         <v/>
       </c>
       <c r="O6" s="23" t="n"/>
-      <c r="P6" s="23" t="n"/>
+      <c r="P6" s="23" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="Q6" s="23" t="n"/>
       <c r="R6" s="23" t="n"/>
       <c r="S6" s="23" t="n"/>
-      <c r="T6" s="23" t="n"/>
+      <c r="T6" s="23" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="U6" s="23">
         <f>IF(AND(O6&lt;&gt;"", OR(P6&lt;&gt;"", Q6&lt;&gt;""), OR(AND(R6&lt;&gt;"", S6&lt;&gt;""), AND(S6&lt;&gt;"", T6&lt;&gt;""), AND(R6&lt;&gt;"", T6&lt;&gt;""))), "Accredited", "In Progress")</f>
         <v/>
       </c>
-      <c r="V6" s="26" t="n"/>
+      <c r="V6" s="26" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="W6" s="23">
         <f>IF(AND(N6="Accredited", U6="Accredited",V6&lt;&gt;""), "Accredited", "In Progress")</f>
         <v/>
@@ -5742,12 +5758,12 @@
       </c>
       <c r="B9" s="27" t="inlineStr">
         <is>
-          <t>thiago.pereira@ish.com.br</t>
+          <t>thiago.goncalves@asper.tec.br</t>
         </is>
       </c>
       <c r="C9" s="27" t="inlineStr">
         <is>
-          <t>ISH</t>
+          <t>Asper</t>
         </is>
       </c>
       <c r="D9" s="27" t="b">
@@ -7025,7 +7041,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D2" t="n">
         <v>21</v>
@@ -7077,10 +7093,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" t="n">
         <v>1</v>
@@ -7356,7 +7372,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D9" t="n">
         <v>4</v>

</xml_diff>

<commit_message>
Corrige célula OT Specialist da Shield (falso positivo legado, sem lastro no Tableau)
Espelha a correção feita em partner-dashboard (commit 32da091).
</commit_message>
<xml_diff>
--- a/data/partner/Focus Partner Tracking BR.xlsx
+++ b/data/partner/Focus Partner Tracking BR.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16960" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BR" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guardian" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tech Certs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="BR" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Guardian" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Tech Certs" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BR'!$A$3:$F$19</definedName>
@@ -1209,11 +1209,7 @@
       </c>
       <c r="Q5" s="23" t="n"/>
       <c r="R5" s="23" t="n"/>
-      <c r="S5" s="23" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="S5" s="23" t="n"/>
       <c r="T5" s="23" t="inlineStr">
         <is>
           <t>OK</t>

</xml_diff>

<commit_message>
chore: certificações EM atualizadas via Tableau (2026-08-12)
</commit_message>
<xml_diff>
--- a/data/partner/Focus Partner Tracking BR.xlsx
+++ b/data/partner/Focus Partner Tracking BR.xlsx
@@ -7143,46 +7143,40 @@
         </is>
       </c>
       <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
         <v>3</v>
       </c>
-      <c r="D4" t="n">
-        <v>6</v>
-      </c>
-      <c r="E4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F4" t="n">
-        <v>4</v>
-      </c>
-      <c r="G4" t="n">
+      <c r="I4" t="n">
         <v>3</v>
       </c>
-      <c r="H4" t="n">
+      <c r="J4" t="n">
+        <v>8</v>
+      </c>
+      <c r="L4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" t="n">
         <v>5</v>
       </c>
-      <c r="I4" t="n">
+      <c r="O4" t="n">
         <v>5</v>
-      </c>
-      <c r="J4" t="n">
-        <v>10</v>
-      </c>
-      <c r="K4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L4" t="n">
-        <v>3</v>
-      </c>
-      <c r="M4" t="n">
-        <v>3</v>
-      </c>
-      <c r="N4" t="n">
-        <v>7</v>
-      </c>
-      <c r="O4" t="n">
-        <v>7</v>
-      </c>
-      <c r="P4" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -7637,46 +7631,46 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D16" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E16" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F16" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G16" t="n">
+        <v>21</v>
+      </c>
+      <c r="H16" t="n">
+        <v>45</v>
+      </c>
+      <c r="I16" t="n">
+        <v>26</v>
+      </c>
+      <c r="J16" t="n">
+        <v>74</v>
+      </c>
+      <c r="K16" t="n">
+        <v>24</v>
+      </c>
+      <c r="L16" t="n">
+        <v>41</v>
+      </c>
+      <c r="M16" t="n">
+        <v>53</v>
+      </c>
+      <c r="N16" t="n">
+        <v>66</v>
+      </c>
+      <c r="O16" t="n">
+        <v>159</v>
+      </c>
+      <c r="P16" t="n">
         <v>20</v>
-      </c>
-      <c r="H16" t="n">
-        <v>44</v>
-      </c>
-      <c r="I16" t="n">
-        <v>25</v>
-      </c>
-      <c r="J16" t="n">
-        <v>73</v>
-      </c>
-      <c r="K16" t="n">
-        <v>23</v>
-      </c>
-      <c r="L16" t="n">
-        <v>40</v>
-      </c>
-      <c r="M16" t="n">
-        <v>52</v>
-      </c>
-      <c r="N16" t="n">
-        <v>65</v>
-      </c>
-      <c r="O16" t="n">
-        <v>158</v>
-      </c>
-      <c r="P16" t="n">
-        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>